<commit_message>
docs: tighten SPM-40 test cases to 16 and record the decisions' sources
Merged overlapping cases (24 -> 16) so each rule is tested once, added the
Approved -> Planning case, and replaced the open questions with the
customer rulings and diagrams each decision rests on. DOCUMENTATION.md:
both Known Gaps rows removed - the status move is built, and the SPM-41
Venue tab lookup bug is being reported to its owner outside this PR.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-40_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-40_Test_Cases.xlsx
@@ -24,14 +24,6 @@
     <sheet name="TC14" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="TC15" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="TC16" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="TC17" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="TC18" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="TC19" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="TC20" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="TC21" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="TC22" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="TC23" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="TC24" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -471,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -543,12 +535,12 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Find a venue opens from the Venues page and lists every active venue when no filter is set</t>
+          <t>Filter by location - and the search page opens on the whole catalogue</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>AC7</t>
+          <t>AC3, AC7</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
@@ -558,7 +550,7 @@
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
@@ -575,12 +567,12 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Filter by location shows only venues in the chosen building</t>
+          <t>Filter by room layout</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>AC3, AC7</t>
+          <t>AC5, AC7</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
@@ -607,12 +599,12 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Location list offers every building that has an active venue</t>
+          <t>Attendance is checked against the chosen layout's capacity, not the venue maximum</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC2, AC5, AC7</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -622,7 +614,7 @@
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
@@ -639,17 +631,17 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Filter by room layout shows only venues offering that layout</t>
+          <t>Attendance exactly at layout capacity matches; one more does not</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>AC5, AC7</t>
+          <t>AC2, AC7</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
@@ -671,22 +663,22 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Filter by expected attendance compares with the chosen layout's capacity, not the venue maximum</t>
+          <t>Attendance of 0 or a fraction is refused</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>AC2, AC5, AC7</t>
+          <t>AC2</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Code</t>
         </is>
       </c>
     </row>
@@ -703,17 +695,17 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Attendance equal to the layout capacity matches; one more does not</t>
+          <t>Filter by accessibility requirements - every ticked one must be met</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>AC2, AC7</t>
+          <t>AC4, AC7</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
@@ -735,22 +727,22 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Expected attendance of 0 or a fraction is refused before searching</t>
+          <t>Filter by required facilities</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>AC2</t>
+          <t>AC6, AC7</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
@@ -767,12 +759,12 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Filter by an accessibility requirement</t>
+          <t>Filter by date and time hides a venue already booked then</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>AC4, AC7</t>
+          <t>AC1, AC7</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -799,12 +791,12 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Several accessibility requirements must ALL be met</t>
+          <t>A venue on hold for another event at that time is hidden</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>AC4, AC7</t>
+          <t>AC1, AC7</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -814,7 +806,7 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Code</t>
         </is>
       </c>
     </row>
@@ -831,22 +823,22 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Filter by required facilities</t>
+          <t>A venue whose setup slot is taken by the next morning's booking is hidden</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>AC6, AC7</t>
+          <t>AC1, AC7</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Code</t>
         </is>
       </c>
     </row>
@@ -863,22 +855,22 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Facilities combine with location</t>
+          <t>Opening hours: starting at opening time matches, one minute earlier does not</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>AC3, AC6, AC7</t>
+          <t>AC1, AC7</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Code</t>
         </is>
       </c>
     </row>
@@ -895,22 +887,22 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Filter by date and time hides a venue already booked at that time</t>
+          <t>A start without an end, or an end not after the start, is refused</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>AC1, AC7</t>
+          <t>AC1</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Code</t>
         </is>
       </c>
     </row>
@@ -927,22 +919,22 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>A venue whose setup slot is taken by the next day's booking is hidden</t>
+          <t>All six filters combined, then Clear filters</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>AC1, AC7</t>
+          <t>AC1, AC2, AC3, AC4, AC5, AC6, AC7</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
@@ -959,12 +951,12 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>A venue blocked for renovation is hidden for those dates</t>
+          <t>Opened from an event, the filters are filled from its requirements - and its own booking does not hide its venue</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>AC1, AC7</t>
+          <t>AC1, AC2, AC4, AC5, AC6, AC7</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -991,12 +983,12 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>A venue on tentative hold for another event at that time is hidden</t>
+          <t>Opening Find a venue for an Approved event moves it to Planning</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>AC1, AC7</t>
+          <t>AC7</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -1023,17 +1015,17 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Opening hours: starting at opening time matches, one minute earlier does not</t>
+          <t>An Event Organiser cannot use venue search</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>AC1, AC7</t>
+          <t>AC7</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
@@ -1042,518 +1034,249 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>TC17</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC17</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>A venue that opens late is hidden for a morning search</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>AC1, AC7</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>TC18</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC18</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="inlineStr">
-        <is>
-          <t>A start without an end, or an end before the start, is refused</t>
-        </is>
-      </c>
-      <c r="D21" s="11" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Acceptance Criterion</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="98.5" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="F21" s="11" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>TC19</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC19</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>Opening Find a venue from an event fills every filter from the event's requirements</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>AC1, AC2, AC4, AC5, AC6</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="F22" s="11" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>TC20</t>
-        </is>
-      </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>SPM-40-TC20</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>The event's own booking does not hide its venue</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>AC1, AC7</t>
-        </is>
-      </c>
+          <t>The Event Coordinator can filter by date and time.</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="9" t="n"/>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="F23" s="11" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>TC21</t>
-        </is>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC21</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="inlineStr">
-        <is>
-          <t>All six filters together return only the venues meeting every one</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="inlineStr">
-        <is>
-          <t>AC1, AC2, AC3, AC4, AC5, AC6, AC7</t>
-        </is>
-      </c>
-      <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="F24" s="11" t="inlineStr">
-        <is>
-          <t>Acceptance Criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>TC22</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC22</t>
-        </is>
-      </c>
-      <c r="C25" s="11" t="inlineStr">
-        <is>
-          <t>Clear filters resets the form and shows the whole catalogue</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="E25" s="11" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="F25" s="11" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>TC23</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC23</t>
-        </is>
-      </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
-          <t>Venue Staff can also use Find a venue</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="E26" s="11" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="F26" s="11" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>TC24</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC24</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>An Event Organiser cannot use venue search</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="E27" s="11" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Acceptance Criterion</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="n"/>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
-        </is>
-      </c>
-      <c r="F30" s="9" t="n"/>
-    </row>
-    <row r="31" ht="139" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>The Event Coordinator can filter by date and time.</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="n"/>
-      <c r="D31" s="9" t="n"/>
-      <c r="E31" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC12
-SPM-40-TC13
-SPM-40-TC14
-SPM-40-TC15
-SPM-40-TC16
-SPM-40-TC17
-SPM-40-TC18
-SPM-40-TC19
-SPM-40-TC20
-SPM-40-TC21</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="n"/>
-    </row>
-    <row r="32" ht="71.5" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>AC2</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>The Event Coordinator can filter by expected attendance/capacity.</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="n"/>
-      <c r="D32" s="9" t="n"/>
-      <c r="E32" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC05
-SPM-40-TC06
-SPM-40-TC07
-SPM-40-TC19
-SPM-40-TC21</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="n"/>
-    </row>
-    <row r="33" ht="58" customHeight="1">
-      <c r="A33" s="11" t="inlineStr">
-        <is>
-          <t>AC3</t>
-        </is>
-      </c>
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>The Event Coordinator can filter by location.</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="n"/>
-      <c r="D33" s="9" t="n"/>
-      <c r="E33" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC02
-SPM-40-TC03
-SPM-40-TC11
-SPM-40-TC21</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="n"/>
-    </row>
-    <row r="34" ht="58" customHeight="1">
-      <c r="A34" s="11" t="inlineStr">
-        <is>
-          <t>AC4</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="inlineStr">
-        <is>
-          <t>The Event Coordinator can filter by accessibility requirements.</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="n"/>
-      <c r="D34" s="9" t="n"/>
-      <c r="E34" s="11" t="inlineStr">
-        <is>
           <t>SPM-40-TC08
-SPM-40-TC09
-SPM-40-TC19
-SPM-40-TC21</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="n"/>
-    </row>
-    <row r="35" ht="58" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
-        <is>
-          <t>AC5</t>
-        </is>
-      </c>
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t>The Event Coordinator can filter by room layout.</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="n"/>
-      <c r="D35" s="9" t="n"/>
-      <c r="E35" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC04
-SPM-40-TC05
-SPM-40-TC19
-SPM-40-TC21</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="n"/>
-    </row>
-    <row r="36" ht="58" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
-        <is>
-          <t>AC6</t>
-        </is>
-      </c>
-      <c r="B36" s="11" t="inlineStr">
-        <is>
-          <t>The Event Coordinator can filter by required facilities.</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="n"/>
-      <c r="D36" s="9" t="n"/>
-      <c r="E36" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC10
-SPM-40-TC11
-SPM-40-TC19
-SPM-40-TC21</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n"/>
-    </row>
-    <row r="37" ht="274" customHeight="1">
-      <c r="A37" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>Results only display venues matching the selected criteria.</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="n"/>
-      <c r="D37" s="9" t="n"/>
-      <c r="E37" s="11" t="inlineStr">
-        <is>
-          <t>SPM-40-TC01
-SPM-40-TC02
-SPM-40-TC04
-SPM-40-TC05
-SPM-40-TC06
-SPM-40-TC08
 SPM-40-TC09
 SPM-40-TC10
 SPM-40-TC11
 SPM-40-TC12
 SPM-40-TC13
+SPM-40-TC14</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n"/>
+    </row>
+    <row r="24" ht="71.5" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>AC2</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>The Event Coordinator can filter by expected attendance/capacity.</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>SPM-40-TC03
+SPM-40-TC04
+SPM-40-TC05
+SPM-40-TC13
+SPM-40-TC14</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="31" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>AC3</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>The Event Coordinator can filter by location.</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>SPM-40-TC01
+SPM-40-TC13</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="44.5" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>AC4</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>The Event Coordinator can filter by accessibility requirements.</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>SPM-40-TC06
+SPM-40-TC13
+SPM-40-TC14</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="58" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>AC5</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>The Event Coordinator can filter by room layout.</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>SPM-40-TC02
+SPM-40-TC03
+SPM-40-TC13
+SPM-40-TC14</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="44.5" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>AC6</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>The Event Coordinator can filter by required facilities.</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>SPM-40-TC07
+SPM-40-TC13
+SPM-40-TC14</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n"/>
+    </row>
+    <row r="29" ht="193" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>AC7</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Results only display venues matching the selected criteria.</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>SPM-40-TC01
+SPM-40-TC02
+SPM-40-TC03
+SPM-40-TC04
+SPM-40-TC06
+SPM-40-TC07
+SPM-40-TC08
+SPM-40-TC09
+SPM-40-TC10
+SPM-40-TC11
+SPM-40-TC13
 SPM-40-TC14
 SPM-40-TC15
-SPM-40-TC16
-SPM-40-TC17
-SPM-40-TC20
-SPM-40-TC21
-SPM-40-TC22
-SPM-40-TC23
-SPM-40-TC24</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n"/>
-    </row>
-    <row r="39" ht="233.5" customHeight="1">
-      <c r="A39" s="7" t="inlineStr">
+SPM-40-TC16</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n"/>
+    </row>
+    <row r="31" ht="233.5" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B39" s="11" t="inlineStr">
-        <is>
-          <t>src/lib/venueSearch.ts
-src/lib/venueSearchForm.ts
-src/lib/validation/venues.ts
-src/app/api/venues/search/route.ts
-src/app/venues/search/page.tsx
-src/app/venues/page.tsx
-src/app/events/[id]/venue/page.tsx
-src/lib/venueSlots.ts
-src/lib/venueSuitability.ts
-src/app/api/venues/route.ts
-src/app/api/facilities/route.ts
-src/app/api/events/[id]/route.ts
-src/lib/permissions.ts
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>UI_DESIGN.md
+design/mockups/VenueSearch.dc.html
 prisma/schema.prisma
 prisma/seed.ts
-design/mockups/VenueSearch.dc.html
-UI_DESIGN.md</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="n"/>
-      <c r="D39" s="8" t="n"/>
-      <c r="E39" s="8" t="n"/>
-      <c r="F39" s="9" t="n"/>
+src/app/api/events/[id]/route.ts
+src/app/api/facilities/route.ts
+src/app/api/venues/route.ts
+src/app/api/venues/search/route.ts
+src/app/events/[id]/venue/page.tsx
+src/app/venues/page.tsx
+src/app/venues/search/page.tsx
+src/lib/permissions.ts
+src/lib/validation/venues.ts
+src/lib/venueSearch.ts
+src/lib/venueSearchForm.ts
+src/lib/venueSlots.ts
+src/lib/venueSuitability.ts</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="B39:F39"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E28:F28"/>
     <mergeCell ref="B1:F1"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B24:D24"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -1572,14 +1295,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1618,7 +1333,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="125.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1626,12 +1341,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page with all filters cleared.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+On the Find a venue page (Venues &gt; Find a venue) with all filters cleared.
+Seed: Marina Grand Hall has an approved booking for 'Straits Medical Research Symposium' (EVT-000004), 09:00-18:00 on its date (72 days after seeding; 8 Dec 2026 if seeded on 28 Sep 2026). Marina Boardroom 2 is under renovation 60-74 days after seeding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1639,12 +1355,13 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Under 'Accessibility requirements', tick 'Braille signage'
-2. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
+          <t>1. Enter From = the symposium's date 09:00, To = the same date 18:00
+2. Choose 'Marina Centre' in 'Location'
+3. Click 'Search'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1652,11 +1369,12 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Accessibility requirements: Braille signage</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>From/To: 8 Dec 2026 09:00-18:00
+Location: Marina Centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1664,8 +1382,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The count reads '2 of 16 venues match'.
-Only Marina Auditorium (MAR-AUD) and One-North Auditorium (ONE-AUD) are listed; on each card 'Braille signage' is shown first, as a green chip.</t>
+          <t>Only Marina Auditorium (MAR-AUD) and Marina Boardroom 1 (MAR-BR1) are listed. Marina Grand Hall (booked) and Marina Boardroom 2 (renovation) are not.</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1495,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1786,9 +1503,9 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page with all filters cleared.
-Orchard Seminar Room has Wheelchair spaces but no Hearing induction loop.</t>
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+On the Find a venue page (Venues &gt; Find a venue) with all filters cleared.
+Seed: Changi Conference Centre has a PENDING booking request for 'Pearl Delta Safety Conference' (EVT-000014), 09:00-17:00, 79 days after seeding (15 Dec 2026 if seeded on 28 Sep 2026).</t>
         </is>
       </c>
     </row>
@@ -1800,8 +1517,8 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Under 'Accessibility requirements', tick 'Wheelchair spaces'
-2. Tick 'Hearing induction loop'
+          <t>1. Choose 'Changi Business Park' in 'Location'
+2. Enter From = the safety conference's date 09:00, To = the same date 17:00
 3. Click 'Search'</t>
         </is>
       </c>
@@ -1814,11 +1531,12 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Accessibility requirements: Wheelchair spaces, Hearing induction loop</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Location: Changi Business Park
+From/To: 15 Dec 2026 09:00-17:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1826,8 +1544,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The count reads '4 of 16 venues match': Changi Conference Centre (CBP-CONF), Marina Auditorium (MAR-AUD), Marina Grand Hall (MAR-GH), One-North Auditorium (ONE-AUD).
-Orchard Seminar Room (ORC-SEM) is not listed although it has wheelchair spaces.</t>
+          <t>Only Changi Meeting Room 1 (CBP-MTG1) and Changi Meeting Room 2 (CBP-MTG2) are listed; Changi Conference Centre is hidden (customer ruling #41: one active hold per venue and time).</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1657,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="125.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1948,12 +1665,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page with all filters cleared.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+On the Find a venue page (Venues &gt; Find a venue) with all filters cleared.
+Seed: Jurong Training Room (JUR-TRN) has an approved booking for 'Harbourline Claims Systems Training' (EVT-000012), 09:00-17:00, 23 days after seeding (20 Oct 2026 if seeded on 28 Sep 2026). It records setup time, so that AM booking also holds the previous day's Night slot (#123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="71.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1961,13 +1679,13 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Under 'Required facilities', tick 'Livestream capability'
-2. Tick 'Green room'
-3. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
+          <t>1. Choose 'Jurong Gateway' in 'Location'
+2. Enter From = the day BEFORE the training 19:00, To = the same day 20:00, and click 'Search'
+3. Change the times to 08:00-11:00 on that same day and click 'Search'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1975,7 +1693,8 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Required facilities: Livestream capability, Green room</t>
+          <t>Location: Jurong Gateway
+From/To: 19 Oct 2026 19:00-20:00, then 08:00-11:00</t>
         </is>
       </c>
     </row>
@@ -1987,8 +1706,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The count reads '3 of 16 venues match': Marina Auditorium (MAR-AUD), Marina Grand Hall (MAR-GH), One-North Auditorium (ONE-AUD).
-On each card the two ticked facilities appear first as green chips.</t>
+          <t>19:00-20:00: only Jurong Skills Lab (JUR-LAB); Jurong Training Room is hidden although nothing is booked in it that evening. (Jurong Expo Floor is under renovation all that week.)
+08:00-11:00: Jurong Skills Lab (JUR-LAB) and Jurong Training Room (JUR-TRN).</t>
         </is>
       </c>
     </row>
@@ -2101,7 +1820,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2109,12 +1828,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page with all filters cleared.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+On the Find a venue page (Venues &gt; Find a venue) with all filters cleared.
+Orchard Hub hours: Seminar Room 08:00-22:00, Studio 08:00-21:00, Gallery 09:00-23:00. 1 Mar 2027 has no bookings there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2122,9 +1842,9 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. In 'Location', choose 'Jurong Gateway'
-2. Under 'Required facilities', tick 'Loading bay access'
-3. Click 'Search'</t>
+          <t>1. Choose 'Orchard Hub' in 'Location'
+2. Enter From = 1 Mar 2027 08:00, To = 1 Mar 2027 22:00, and click 'Search'
+3. Change From to 07:59 and click 'Search'</t>
         </is>
       </c>
     </row>
@@ -2136,12 +1856,12 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Location: Jurong Gateway
-Required facilities: Loading bay access</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>Location: Orchard Hub
+From/To: 1 Mar 2027 08:00-22:00, then 07:59-22:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2149,7 +1869,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Only Jurong Expo Floor (JUR-EXP) and Jurong Skills Lab (JUR-LAB) are listed. Marina Grand Hall and Orchard Gallery also have a loading bay but are in other buildings, so they are not shown.</t>
+          <t>08:00-22:00: only Orchard Seminar Room (ORC-SEM).
+07:59-22:00: no venues; 'No venues match these filters' is shown.</t>
         </is>
       </c>
     </row>
@@ -2262,7 +1983,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2270,13 +1991,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-Seed data: Marina Grand Hall (MAR-GH) has an approved booking for 'Straits Medical Research Symposium' (EVT-000004), 09:00-18:00 on its event date (72 days after seeding; 8 Dec 2026 if seeded on 28 Sep 2026).
-On the Find a venue page with all filters cleared (opened from the Venues page, not from an event).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+On the Find a venue page (Venues &gt; Find a venue) with all filters cleared.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2284,14 +2004,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. In 'From', enter the symposium's date at 09:00
-2. In 'To', enter the same date at 18:00
-3. In 'Location', choose 'Marina Centre'
-4. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
+          <t>1. Enter From = 1 Mar 2027 09:00, leave 'To' empty, and click 'Search'
+2. Enter To = 1 Mar 2027 09:00 and click 'Search'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2299,9 +2017,8 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>From: 8 Dec 2026 09:00
-To: 8 Dec 2026 18:00
-Location: Marina Centre</t>
+          <t>From: 1 Mar 2027 09:00
+To: empty, then 1 Mar 2027 09:00</t>
         </is>
       </c>
     </row>
@@ -2313,8 +2030,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Marina Grand Hall (MAR-GH) is not listed.
-Marina Auditorium (MAR-AUD) and Marina Boardroom 1 (MAR-BR1) are listed. Marina Boardroom 2 (MAR-BR2) is also missing - it is under renovation that day (see TC14).</t>
+          <t>First: 'To' shows 'Give both a start and an end, or clear both.'
+Second: 'To' shows 'The end must be after the start.'
+The results do not change either time.</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2145,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="125.5" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2435,13 +2153,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-Seed data: Jurong Training Room (JUR-TRN) has an approved booking for 'Harbourline Claims Systems Training' (EVT-000012), 09:00-17:00, 23 days after seeding (20 Oct 2026 if seeded on 28 Sep 2026). JUR-TRN records setup time, so under the customer's slot rules (#123) that AM booking also takes the previous day's Night slot.
-On the Find a venue page with all filters cleared.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="85" customHeight="1">
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+On the Find a venue page (Venues &gt; Find a venue) with all filters cleared.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="125.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2449,15 +2166,17 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. In 'Location', choose 'Jurong Gateway'
-2. Enter From = the day BEFORE the training at 19:00, To = the same day at 20:00
-3. Click 'Search'
-4. Change From to 08:00 and To to 11:00 on that same day
-5. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
+          <t>1. Enter From = 1 Mar 2027 09:00, To = 1 Mar 2027 12:00
+2. Enter 100 in 'Expected attendance'
+3. Choose 'Marina Centre' in 'Location' and 'Theatre' in 'Room layout'
+4. Tick 'Step-free access' and 'Hearing induction loop' under Accessibility requirements
+5. Tick 'Built-in PA system' under Required facilities
+6. Click 'Search'
+7. Click 'Clear filters'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="85" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2465,8 +2184,12 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Location: Jurong Gateway
-From/To: 19 Oct 2026 19:00-20:00, then 19 Oct 2026 08:00-11:00</t>
+          <t>From/To: 1 Mar 2027 09:00-12:00
+Expected attendance: 100
+Location: Marina Centre
+Room layout: Theatre
+Accessibility: Step-free access, Hearing induction loop
+Facilities: Built-in PA system</t>
         </is>
       </c>
     </row>
@@ -2478,8 +2201,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>19:00-20:00: only Jurong Skills Lab (JUR-LAB) is listed. Jurong Training Room is hidden although nothing is booked in it that evening - the Night slot is its next-morning setup.
-08:00-11:00: Jurong Skills Lab (JUR-LAB) and Jurong Training Room (JUR-TRN) are both listed.</t>
+          <t>After Search: only Marina Auditorium (MAR-AUD, theatre 220) then Marina Grand Hall (MAR-GH, theatre 500); the Theatre capacity is bold and the three ticked items are green chips.
+After Clear filters: every filter is empty and '16 of 16 venues match'.</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2315,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="85" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2600,13 +2323,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-Seed data: Jurong Expo Floor (JUR-EXP) is unavailable for renovation from 21 to 28 days after seeding (19-26 Oct 2026 if seeded on 28 Sep 2026).
-On the Find a venue page with all filters cleared.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="85" customHeight="1">
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123). He coordinates 'Straits Medical Research Symposium' (EVT-000004, status Planning), booked into Marina Grand Hall.
+The symposium: 200 people, Theatre, 09:00-18:00; mandatory High-density WiFi, Video conferencing suite, Livestream capability, Hearing induction loop, Wheelchair spaces; nice-to-have Catering pantry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2614,15 +2336,13 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. In 'Location', choose 'Jurong Gateway'
-2. Enter From = 22 days after seeding at 09:00, To = the same day at 12:00
-3. Click 'Search'
-4. Change From/To to 1 Mar 2027 09:00-12:00
-5. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
+          <t>1. Open the symposium from Events
+2. Click the 'Venue' tab
+3. Click 'Search with filters'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2630,12 +2350,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Location: Jurong Gateway
-From/To: 20 Oct 2026 09:00-12:00, then 1 Mar 2027 09:00-12:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44.5" customHeight="1">
+          <t>Event: EVT-000004</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="179.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2643,8 +2362,10 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>20 Oct: Jurong Expo Floor (JUR-EXP) is not listed.
-1 Mar 2027: Jurong Expo Floor (JUR-EXP) is listed again, with Jurong Skills Lab and Jurong Training Room.</t>
+          <t>Find a venue opens with breadcrumb 'Events / EVT-000004 / Find a venue' and the subtitle 'Filled in from Straits Medical Research Symposium's requirements...'.
+From/To = its date 09:00 / 18:00; Expected attendance 200; Room layout Theatre; Location 'Any building'. Wheelchair spaces and Hearing induction loop are ticked, and so are High-density WiFi, Video conferencing suite and Livestream capability; Catering pantry is NOT ticked.
+Results: Marina Auditorium (MAR-AUD), Changi Conference Centre (CBP-CONF), Marina Grand Hall (MAR-GH) - Marina Grand Hall IS listed because its booking is this event's own (compare TC08). Each card has 'Check suitability'.
+No status message appears and the event stays in Planning.</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2478,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="98.5" customHeight="1">
+    <row r="3" ht="71.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2765,13 +2486,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-Seed data: Changi Conference Centre (CBP-CONF) has a PENDING booking request for 'Pearl Delta Safety Conference' (EVT-000014), 09:00-17:00, 79 days after seeding (15 Dec 2026 if seeded on 28 Sep 2026).
-On the Find a venue page with all filters cleared.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+Seed: 'SPM40 Approved Workshop' (status Approved, coordinator Daniel Tan, 30 people, Classroom, 09:00-12:00, 180 days after seeding) - the only Approved event in the seed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="71.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2779,13 +2499,14 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. In 'Location', choose 'Changi Business Park'
-2. Enter From = the safety conference's date at 09:00, To = the same date at 17:00
-3. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+          <t>1. Open 'SPM40 Approved Workshop' from Events and note its status badge
+2. Click the 'Venue' tab, then 'Search with filters'
+3. Go back to the event's Overview
+4. Reopen Find a venue from the Venue tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2793,12 +2514,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Location: Changi Business Park
-From/To: 15 Dec 2026 09:00-17:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>Event: SPM40 Approved Workshop</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="112" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2806,7 +2526,10 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Only Changi Meeting Room 1 (CBP-MTG1) and Changi Meeting Room 2 (CBP-MTG2) are listed. Changi Conference Centre is hidden because it is already on hold for that time (customer ruling #41: one active hold per venue and time).</t>
+          <t>Before: the status badge reads 'Approved'.
+Find a venue shows the green message 'Planning has started - This event has moved from Approved to Planning now that its venue search has begun.' above the filters, with results already listed.
+Back on the Overview the status badge reads 'Planning'.
+Reopening Find a venue shows no message and the status stays Planning.</t>
         </is>
       </c>
     </row>
@@ -2919,7 +2642,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2927,13 +2650,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page with all filters cleared.
-Orchard Seminar Room is open 08:00-22:00; Orchard Studio 08:00-21:00; Orchard Gallery 09:00-23:00.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="71.5" customHeight="1">
+          <t>Logged in as Event Organiser Evelyn Chen (email in npx prisma studio &gt; users; password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="31" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2941,15 +2662,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. In 'Location', choose 'Orchard Hub'
-2. Enter From = 1 Mar 2027 08:00, To = 1 Mar 2027 22:00
-3. Click 'Search'
-4. Change From to 07:59
-5. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+          <t>1. Check the sidebar for 'Venues'
+2. Type /venues/search into the address bar and press Enter</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2957,12 +2675,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Location: Orchard Hub
-From/To: 1 Mar 2027 08:00-22:00, then 07:59-22:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>Page: /venues/search</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2970,173 +2687,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>08:00-22:00: only Orchard Seminar Room (ORC-SEM) is listed (the Studio closes at 21:00, the Gallery opens at 09:00).
-07:59-22:00: no venue is listed; 'No venues match these filters' is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>kayalvizhi24</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46293</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-40-TC17</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="58" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page with all filters cleared.
-One-North Rooftop Terrace opens at 16:00.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="71.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. In 'Location', choose 'One-North'
-2. Enter From = 1 Mar 2027 09:00, To = 1 Mar 2027 11:00
-3. Click 'Search'
-4. Change From to 17:00 and To to 22:00
-5. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Location: One-North
-From/To: 1 Mar 2027 09:00-11:00, then 17:00-22:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>09:00-11:00: One-North Auditorium (ONE-AUD) and One-North Seminar Room (ONE-SEM) are listed; One-North Rooftop Terrace is not.
-17:00-22:00: One-North Auditorium (ONE-AUD) and One-North Rooftop Terrace (ONE-ROOF) are listed (the Seminar Room closes at 21:00).</t>
+          <t>The sidebar has no 'Venues' link.
+The page shows 'Not available - Venue search is for ConnectSphere staff.' and no venues.</t>
         </is>
       </c>
     </row>
@@ -3247,13 +2799,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="98.5" customHeight="1">
+    <row r="2" ht="31" customHeight="1">
       <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Approved -&gt; Planning: the status lifecycle diagram labels this move 'search', and the seed's status history reason for Planning is 'Venue search started'. SPM-40 does NOT change the event's status - searching is read-only, and an event would flip to Planning just because someone looked. Nothing else moves Approved -&gt; Planning yet either. Should the move happen when the coordinator submits the first venue booking request (SPM-42), or when they first open Find a venue for the event?</t>
+          <t>Decided from existing documentation, recorded here so reviewers can check the source rather than asking again:</t>
         </is>
       </c>
       <c r="C2" s="11" t="n"/>
@@ -3264,62 +2816,62 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Tentative holds (#41): a venue with a PENDING booking request for another event at an overlapping time is hidden from results, because the customer allows only one active hold per venue and time, so asking for it would only be refused. SPM-46's availability calendar shows the same hold as a warning rather than a block. Confirm hiding it is right for search.</t>
+          <t>(1) Opening Find a venue for an Approved event moves it to Planning (TC15) - the status lifecycle diagram labels Approved -&gt; Planning 'search', the BPMN puts 'Search venues &amp; check suitability' right after approval, and the seed's history reason for Planning is 'Venue search started'. Only the assigned coordinator triggers it, and only from Approved.</t>
         </is>
       </c>
       <c r="C3" s="11" t="n"/>
     </row>
-    <row r="4" ht="71.5" customHeight="1">
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="11" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Opening hours: a venue is matched only when the search starts at or after its opening time and ends at or before its closing time (checked on the first and last day of a multi-day search, not overnight). The AC says 'date and time' only; this is the team's reading of #46 (Venue Staff maintain operating hours). Confirm.</t>
+          <t>(2) Another event's pending booking request hides a venue (TC09) - #41: only one active tentative hold or confirmed booking per venue and overlapping time.</t>
         </is>
       </c>
       <c r="C4" s="11" t="n"/>
     </row>
-    <row r="5" ht="85" customHeight="1">
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="11" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Setup and turnaround: under the customer's slot rules (#50, #107, #108, #123, implemented by SPM-46's venueSlots.ts) the searched event's OWN setup and turnaround slots must be free too, so e.g. an AM search hides a venue whose previous-night slot is another booking's turnaround. This makes the search stricter than 'is anything booked during my hours'. Confirm this is wanted.</t>
+          <t>(3) The searched event's own setup and turnaround slots must be free too (TC10) - #123: 'venue availability and booking-conflict checking reflect these rules'.</t>
         </is>
       </c>
       <c r="C5" s="11" t="n"/>
     </row>
-    <row r="6" ht="44.5" customHeight="1">
+    <row r="6" ht="31" customHeight="1">
       <c r="A6" s="11" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Attendance with no layout chosen matches a venue if ANY of its layouts seats that many; a venue with no layouts never matches an attendance filter. Venue.maxCapacity is never used (#112). Confirm.</t>
+          <t>(4) The venue must be open for the requested hours (TC11) - #46: Venue Staff maintain operating hours, all days equal.</t>
         </is>
       </c>
       <c r="C6" s="11" t="n"/>
     </row>
-    <row r="7" ht="71.5" customHeight="1">
+    <row r="7" ht="31" customHeight="1">
       <c r="A7" s="11" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Pre-filling from an event ticks only its MANDATORY facility and accessibility requirements; nice-to-haves are left unticked so they don't hide venues (AC7 would drop any venue lacking one). Location is left as 'Any building' because an event has no location requirement. Confirm both.</t>
+          <t>(5) Attendance with no layout chosen matches if any layout seats everyone; Venue.maxCapacity is never used (TC03) - #112, #119.</t>
         </is>
       </c>
       <c r="C7" s="11" t="n"/>
     </row>
-    <row r="8" ht="71.5" customHeight="1">
+    <row r="8" ht="44.5" customHeight="1">
       <c r="A8" s="11" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Mockup vs AC7: design/mockups/VenueSearch.dc.html shows over-capacity, partial-match and unavailable venues greyed out in the list. AC7 says results show ONLY matching venues, so SPM-40 hides them; the greyed 'not suitable, and why' view is SPM-41's Venue tab. The mockup should be updated or the team should confirm the split.</t>
+          <t>(6) Pre-fill ticks mandatory requirements only and leaves Location as 'Any building' (TC14) - EventFacilityRequirement.isMandatory 'must NOT disqualify a venue'; #80; #111.</t>
         </is>
       </c>
       <c r="C8" s="11" t="n"/>
@@ -3330,7 +2882,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>No 'Request' button: the mockup's Request / Request anyway buttons belong to S-15 Venue booking request (SPM-42), not built. SPM-40 offers 'Check suitability' (SPM-41) from an event's results instead.</t>
+          <t>(7) Non-matching venues are hidden, not greyed as in design/mockups/VenueSearch.dc.html - AC7 and #83; the greyed view is SPM-41's Venue tab.</t>
         </is>
       </c>
       <c r="C9" s="11" t="n"/>
@@ -3341,1161 +2893,24 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Dates in these test cases depend on the day the seed was run - seed dates are relative to 'today'. Absolute dates given assume seeding on 28 Sep 2026; recompute from the event dates shown in the app otherwise.</t>
+          <t>Not decisions: there is no 'Request' button because S-15 venue booking (SPM-42) is not built; and seed dates are relative to the day the seed ran - absolute dates here assume seeding on 28 Sep 2026.</t>
         </is>
       </c>
       <c r="C10" s="11" t="n"/>
     </row>
-    <row r="11" ht="112" customHeight="1">
+    <row r="11" ht="71.5" customHeight="1">
       <c r="A11" s="11" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Found while testing, outside SPM-40: on main, the SPM-41 Venue tab (/events/EVT-000004/venue) always says the event does not exist, because GET /api/events/[id]/venue-suitability looks the event up by its internal id while every link now uses the EVT- reference (SPM-31). TC19 reaches Find a venue through that tab's 'Search with filters' button, which still works because the button renders even when the tab's own check fails. The SPM-41 owner should switch that route to parseEventReference().</t>
+          <t>Known, outside SPM-40: the SPM-41 Venue tab currently says the event does not exist for every event (its route looks events up by internal id, but links use the EVT- reference since SPM-31). TC14 and TC15 still work because the 'Search with filters' button renders above that message. Reported to the SPM-41 owner separately.</t>
         </is>
       </c>
       <c r="C11" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-40-TC18</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page with all filters cleared.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Enter From = 1 Mar 2027 09:00 and leave 'To' empty
-2. Click 'Search'
-3. Enter To = 1 Mar 2027 09:00
-4. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>From: 1 Mar 2027 09:00
-To: (empty), then 1 Mar 2027 09:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>First search: 'To' shows 'Give both a start and an end, or clear both.' and the results do not change.
-Second search: 'To' shows 'The end must be after the start.' and the results do not change.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>kayalvizhi24</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46293</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-40-TC19</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="112" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123), coordinator of 'Straits Medical Research Symposium' (EVT-000004, status Planning).
-The symposium expects 200 people, theatre layout, 09:00-18:00 on its date; mandatory requirements: High-density WiFi, Video conferencing suite, Livestream capability, Hearing induction loop, Wheelchair spaces; Catering pantry is a nice-to-have.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Open 'Straits Medical Research Symposium' from Events
-2. Click the 'Venue' tab
-3. Click 'Search with filters'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Event: EVT-000004</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="166" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>The Find a venue page opens with the breadcrumb 'Events / EVT-000004 / Find a venue' and the subtitle 'Filled in from Straits Medical Research Symposium's requirements...'.
-From/To show the event's date 09:00 and 18:00; Expected attendance 200; Room layout Theatre; Location 'Any building'.
-Wheelchair spaces and Hearing induction loop are ticked under Accessibility requirements; High-density WiFi, Video conferencing suite and Livestream capability are ticked under Required facilities; Catering pantry is NOT ticked.
-The results are already shown: Marina Auditorium (MAR-AUD), Changi Conference Centre (CBP-CONF), Marina Grand Hall (MAR-GH), each with a 'Check suitability' button.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>kayalvizhi24</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46293</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-40-TC20</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="58" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>As TC19: Marina Grand Hall is booked (approved) for the symposium itself.
-Find a venue opened from the symposium's Venue tab (filters pre-filled).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="71.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Look for Marina Grand Hall in the results
-2. Click 'Venues' in the sidebar, then 'Find a venue'
-3. Enter the same From/To, Expected attendance 200, Room layout Theatre, and tick the same five requirements as TC19
-4. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>From/To: symposium date 09:00-18:00
-Expected attendance: 200
-Room layout: Theatre</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Opened from the event: Marina Grand Hall (MAR-GH) IS listed - its only booking that day is this event's own.
-Opened from Venues (no event): Marina Grand Hall is NOT listed; only Marina Auditorium (MAR-AUD) and Changi Conference Centre (CBP-CONF) are.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>kayalvizhi24</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46293</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-40-TC21</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page with all filters cleared.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="112" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Enter From = 1 Mar 2027 09:00, To = 1 Mar 2027 12:00
-2. Enter 100 in 'Expected attendance'
-3. Choose 'Marina Centre' in 'Location'
-4. Choose 'Theatre' in 'Room layout'
-5. Tick 'Step-free access' and 'Hearing induction loop' under Accessibility requirements
-6. Tick 'Built-in PA system' under Required facilities
-7. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="85" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>From/To: 1 Mar 2027 09:00-12:00
-Expected attendance: 100
-Location: Marina Centre
-Room layout: Theatre
-Accessibility: Step-free access, Hearing induction loop
-Facilities: Built-in PA system</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Only Marina Auditorium (MAR-AUD, theatre 220) and Marina Grand Hall (MAR-GH, theatre 500) are listed, in that order.
-The Theatre capacity is shown in bold on each card, and the three ticked items appear first as green chips.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>kayalvizhi24</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46293</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-40-TC22</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page after running TC21.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="17.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Click 'Clear filters'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="31" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Every filter is empty again ('Any building', 'Any layout', no boxes ticked) and the count reads '16 of 16 venues match'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>kayalvizhi24</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46293</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-40-TC23</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="31" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Logged in as Venue Staff Marcus Wong (marcus.wong@connectsphere.com / password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Click 'Venues' in the sidebar
-2. Click 'Find a venue'
-3. Choose 'Orchard Hub' in 'Location' and click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Location: Orchard Hub</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>On the Venues page 'Find a venue' sits beside 'Add venue'.
-The search lists Orchard Gallery (ORC-GAL), Orchard Seminar Room (ORC-SEM) and Orchard Studio (ORC-STU). Retired venues never appear in the results.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>kayalvizhi24</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46293</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-40-TC24</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Logged in as Event Organiser Evelyn Chen (look up her email in npx prisma studio &gt; users; password123), organiser of 'Straits Medical Research Symposium'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="31" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Check the sidebar for a 'Venues' link
-2. Type /venues/search into the address bar and press Enter</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Page: /venues/search</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>There is no 'Venues' link in the organiser's sidebar.
-The page shows the error 'Not available - Venue search is for ConnectSphere staff.' and no venue is listed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>kayalvizhi24</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46293</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -4540,12 +2955,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed data freshly loaded (npx prisma db seed): 16 active venues.
+          <t>Seed data freshly loaded (npx prisma db seed): 16 active venues in 5 buildings.
 Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="44.5" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -4553,9 +2968,10 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Venues' in the sidebar
-2. Click 'Find a venue'
-3. Look at the results count above the list</t>
+          <t>1. Click 'Venues' in the sidebar, then 'Find a venue'
+2. Note the results count
+3. Open the 'Location' dropdown
+4. Choose 'Marina Centre' and click 'Search'</t>
         </is>
       </c>
     </row>
@@ -4567,11 +2983,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>No filters set</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="98.5" customHeight="1">
+          <t>Location: Marina Centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="112" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -4579,9 +2995,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The 'Find a venue' page opens with the subtitle 'Only venues matching every filter you set are shown.'
-All filters are empty ('Any building', 'Any layout', no boxes ticked).
-The count reads '16 of 16 venues match' and 16 venue cards are listed, from Changi Conference Centre (CBP-CONF) to Orchard Studio (ORC-STU).</t>
+          <t>The page opens with every filter empty and '16 of 16 venues match'.
+Location offers 'Any building', Changi Business Park, Jurong Gateway, Marina Centre, One-North, Orchard Hub.
+After searching: '4 of 16 venues match' - only Marina Auditorium (MAR-AUD), Marina Boardroom 1 (MAR-BR1), Marina Boardroom 2 (MAR-BR2) and Marina Grand Hall (MAR-GH), each showing 'Marina Centre'.</t>
         </is>
       </c>
     </row>
@@ -4694,7 +3110,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -4702,8 +3118,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page with all filters cleared.</t>
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+On the Find a venue page (Venues &gt; Find a venue) with all filters cleared.</t>
         </is>
       </c>
     </row>
@@ -4715,7 +3131,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. In 'Location', choose 'Marina Centre'
+          <t>1. In 'Room layout', choose 'Banquet'
 2. Click 'Search'</t>
         </is>
       </c>
@@ -4728,11 +3144,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Location: Marina Centre</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Room layout: Banquet</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -4740,8 +3156,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The count reads '4 of 16 venues match'.
-Only Marina Auditorium (MAR-AUD), Marina Boardroom 1 (MAR-BR1), Marina Boardroom 2 (MAR-BR2) and Marina Grand Hall (MAR-GH) are listed; each card shows 'Marina Centre' as its building.</t>
+          <t>'5 of 16 venues match': Changi Conference Centre (CBP-CONF), Jurong Expo Floor (JUR-EXP), Marina Grand Hall (MAR-GH), One-North Rooftop Terrace (ONE-ROOF), Orchard Gallery (ORC-GAL). 'Banquet' appears in each card's layout line.</t>
         </is>
       </c>
     </row>
@@ -4854,7 +3269,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="71.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -4862,12 +3277,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+On the Find a venue page (Venues &gt; Find a venue) with all filters cleared.
+Marina Grand Hall: maximum 500, theatre 500, classroom 250.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -4875,13 +3291,14 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the 'Location' dropdown
-2. Choose 'Jurong Gateway' and click 'Search'
-3. Open the 'Location' dropdown again</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
+          <t>1. Enter 300 in 'Expected attendance'
+2. Click 'Search'
+3. Choose 'Classroom' in 'Room layout'
+4. Click 'Search'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -4889,11 +3306,12 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Location: Jurong Gateway</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Expected attendance: 300
+Room layout: any, then Classroom</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -4901,8 +3319,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The dropdown lists 'Any building', Changi Business Park, Jurong Gateway, Marina Centre, One-North, Orchard Hub.
-After searching Jurong Gateway (3 of 16 match: JUR-EXP, JUR-LAB, JUR-TRN), the dropdown still lists all five buildings - picking one does not remove the others.</t>
+          <t>Any layout: '2 of 16 venues match' - Marina Grand Hall (MAR-GH) first, then Jurong Expo Floor (JUR-EXP) (smallest room that fits first).
+Classroom: '0 of 16 venues match' with 'No venues match these filters' and 'Try a wider time, a different layout or location, or fewer facilities.' Marina Grand Hall is not shown although its maximum is 500.</t>
         </is>
       </c>
     </row>
@@ -5015,7 +3433,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -5023,12 +3441,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page with all filters cleared.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="31" customHeight="1">
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+On the Find a venue page (Venues &gt; Find a venue) with all filters cleared.
+Theatre capacity: Marina Grand Hall 500, Jurong Expo Floor 600.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -5036,12 +3455,13 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. In 'Room layout', choose 'Banquet'
-2. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
+          <t>1. Choose 'Theatre' in 'Room layout'
+2. Enter 500 in 'Expected attendance' and click 'Search'
+3. Change 'Expected attendance' to 501 and click 'Search'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -5049,11 +3469,12 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Room layout: Banquet</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Room layout: Theatre
+Expected attendance: 500, then 501</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -5061,8 +3482,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The count reads '5 of 16 venues match'.
-Only Changi Conference Centre (CBP-CONF), Jurong Expo Floor (JUR-EXP), Marina Grand Hall (MAR-GH), One-North Rooftop Terrace (ONE-ROOF) and Orchard Gallery (ORC-GAL) are listed, and 'Banquet' appears in each card's layout line.</t>
+          <t>500: Marina Grand Hall (MAR-GH) and Jurong Expo Floor (JUR-EXP).
+501: only Jurong Expo Floor (JUR-EXP).</t>
         </is>
       </c>
     </row>
@@ -5175,7 +3596,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -5183,13 +3604,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page with all filters cleared.
-Marina Grand Hall seats 500 theatre-style but 250 classroom-style.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+On the Find a venue page (Venues &gt; Find a venue) with all filters cleared.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="31" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -5197,14 +3617,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Enter 300 in 'Expected attendance'
-2. Click 'Search'
-3. Choose 'Classroom' in 'Room layout'
-4. Click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+          <t>1. Enter 0 in 'Expected attendance' and click 'Search'
+2. Change it to 12.5 and click 'Search'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -5212,12 +3630,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Expected attendance: 300
-Room layout: (any), then Classroom</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="112" customHeight="1">
+          <t>Expected attendance: 0, then 12.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -5225,8 +3642,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>With any layout: '2 of 16 venues match' - Marina Grand Hall (MAR-GH) then Jurong Expo Floor (JUR-EXP); the smallest room that still fits is listed first.
-With Classroom: '0 of 16 venues match' and the message 'No venues match these filters' with 'Try a wider time, a different layout or location, or fewer facilities.' No venue seats 300 in classroom layout, so Marina Grand Hall (classroom 250) is not shown even though its maximum is 500.</t>
+          <t>Both times the field shows 'Enter a whole number of people, 1 or more.' and the results do not change.</t>
         </is>
       </c>
     </row>
@@ -5339,7 +3755,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -5347,13 +3763,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page with all filters cleared.
-Marina Grand Hall theatre capacity 500; Jurong Expo Floor theatre capacity 600.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="71.5" customHeight="1">
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+On the Find a venue page (Venues &gt; Find a venue) with all filters cleared.
+Orchard Seminar Room has Wheelchair spaces but no Hearing induction loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -5361,11 +3777,8 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Choose 'Theatre' in 'Room layout'
-2. Enter 500 in 'Expected attendance'
-3. Click 'Search'
-4. Change 'Expected attendance' to 501
-5. Click 'Search'</t>
+          <t>1. Under 'Accessibility requirements', tick 'Wheelchair spaces' and 'Hearing induction loop'
+2. Click 'Search'</t>
         </is>
       </c>
     </row>
@@ -5377,12 +3790,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Room layout: Theatre
-Expected attendance: 500, then 501</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44.5" customHeight="1">
+          <t>Accessibility requirements: Wheelchair spaces, Hearing induction loop</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -5390,8 +3802,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>At 500: Marina Grand Hall (MAR-GH) and Jurong Expo Floor (JUR-EXP) are listed, Marina first.
-At 501: only Jurong Expo Floor (JUR-EXP) is listed.</t>
+          <t>'4 of 16 venues match': Changi Conference Centre (CBP-CONF), Marina Auditorium (MAR-AUD), Marina Grand Hall (MAR-GH), One-North Auditorium (ONE-AUD); both ticked items appear first on each card as green chips.
+Orchard Seminar Room (ORC-SEM) is not listed.</t>
         </is>
       </c>
     </row>
@@ -5504,7 +3916,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -5512,12 +3924,12 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).
-On the Find a venue page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
+          <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
+On the Find a venue page (Venues &gt; Find a venue) with all filters cleared.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -5525,10 +3937,8 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Enter 0 in 'Expected attendance'
-2. Click 'Search'
-3. Change 'Expected attendance' to 12.5
-4. Click 'Search'</t>
+          <t>1. Under 'Required facilities', tick 'Livestream capability' and 'Green room'
+2. Click 'Search'</t>
         </is>
       </c>
     </row>
@@ -5540,11 +3950,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Expected attendance: 0, then 12.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="31" customHeight="1">
+          <t>Required facilities: Livestream capability, Green room</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -5552,7 +3962,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Both times the field shows 'Enter a whole number of people, 1 or more.' in red and the results list does not change.</t>
+          <t>'3 of 16 venues match': Marina Auditorium (MAR-AUD), Marina Grand Hall (MAR-GH), One-North Auditorium (ONE-AUD); the two ticked facilities appear first on each card as green chips.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SPM-40: test cases re-checked on the fixed seed and the topped-up data
All 16 expected results match the live search API on the shared database.
No overlaps found, so no cases added or removed. TC01 no longer asks for a
fresh reseed, TC15 says how to reset its event (topup script), and TC16
names Evelyn Chen's login instead of pointing at Prisma Studio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-40_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-40_Test_Cases.xlsx
@@ -490,7 +490,6 @@
       <c r="E1" s="8" t="n"/>
       <c r="F1" s="9" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -1035,8 +1034,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
@@ -1228,7 +1225,6 @@
       </c>
       <c r="F29" s="9" t="n"/>
     </row>
-    <row r="30"/>
     <row r="31" ht="233.5" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
         <is>
@@ -1265,8 +1261,8 @@
   <mergeCells count="18">
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="E29:F29"/>
+    <mergeCell ref="B23:D23"/>
     <mergeCell ref="E24:F24"/>
-    <mergeCell ref="B23:D23"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="E25:F25"/>
     <mergeCell ref="B26:D26"/>
@@ -1412,7 +1408,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -1500,7 +1495,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="98.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1575,7 +1570,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -1739,7 +1733,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -1903,7 +1896,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2066,7 +2058,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2237,7 +2228,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2401,7 +2391,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2489,7 +2478,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2498,7 +2487,7 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
-Seed: 'SPM40 Approved Workshop' (status Approved, coordinator Daniel Tan, 30 people, Classroom, 09:00-12:00 on 25 Mar 2027, day 180 of the fixed 2026-09-26 seed) - the only Approved event in the seed.</t>
+Seed: 'SPM40 Approved Workshop' (status Approved, coordinator Daniel Tan, 30 people, Classroom, 09:00-12:00 on 25 Mar 2027, day 180 of the fixed 2026-09-26 seed) - the only Approved event in the seed. If it is missing, or already in Planning because this case was run before, run: npx tsx prisma/topup-spm40-46.ts (adds or resets it without a reseed).</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2555,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2662,7 +2650,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Logged in as Event Organiser Evelyn Chen (email in npx prisma studio &gt; users; password123).</t>
+          <t>Logged in as Event Organiser Evelyn Chen: evelyn.chen@straitsmedic.com / password123</t>
         </is>
       </c>
     </row>
@@ -2726,7 +2714,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2900,7 +2887,7 @@
       </c>
       <c r="C9" s="11" t="n"/>
     </row>
-    <row r="10" ht="44.5" customHeight="1">
+    <row r="10" ht="58" customHeight="1">
       <c r="A10" s="11" t="n">
         <v>9</v>
       </c>
@@ -2960,7 +2947,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="71.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2968,7 +2955,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Seed data freshly loaded (npx prisma db seed): 16 active venues in 5 buildings.
+          <t>Demo data from prisma/seed.ts: 16 active venues in 5 buildings. A venue retired while testing (e.g. by SPM-46-TC14) must be restored first.
 Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
         </is>
       </c>
@@ -3036,7 +3023,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3196,7 +3182,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3361,7 +3346,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3525,7 +3509,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3685,7 +3668,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3847,7 +3829,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -4007,7 +3988,6 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
SPM-40-TC05: expect the browser's own validation message
The attendance box is type=number with min=1 and the form has no
noValidate, so the browser blocks 0 and 12.5 before the page's own check
runs. The expected result now describes what the tester actually sees.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-40_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-40_Test_Cases.xlsx
@@ -3634,7 +3634,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="31" customHeight="1">
+    <row r="6" ht="98.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3642,7 +3642,10 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Both times the field shows 'Enter a whole number of people, 1 or more.' and the results do not change.</t>
+          <t>Both times the browser stops the search before it is sent and points at 'Expected attendance' with its own message (wording varies by browser; in Chrome):
+0: 'Value must be greater than or equal to 1.'
+12.5: 'Please enter a valid value. The two nearest valid values are 12 and 13.'
+The results do not change either time.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SPM-40 test cases: give typed times in 24-hour with the 12-hour form
The From/To boxes are drawn by the browser, which shows 12- or 24-hour by
the tester's locale; the app itself displays 24-hour. Each typed time now
reads e.g. '09:00 (9:00 am)', and From/To are separate lines with a date.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-40_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-40_Test_Cases.xlsx
@@ -1355,13 +1355,13 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Enter From = the symposium's date 09:00, To = the same date 18:00
+          <t>1. Enter From = the symposium's date, 09:00 (9:00 am), To = the same date, 18:00 (6:00 pm)
 2. Choose 'Marina Centre' in 'Location'
 3. Click 'Search'</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="31" customHeight="1">
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1369,7 +1369,8 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>From/To: 7 Dec 2026 09:00-18:00
+          <t>From: 7 Dec 2026, 09:00 (9:00 am)
+To: 7 Dec 2026, 18:00 (6:00 pm)
 Location: Marina Centre</t>
         </is>
       </c>
@@ -1518,12 +1519,12 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Choose 'Changi Business Park' in 'Location'
-2. Enter From = the safety conference's date 09:00, To = the same date 17:00
+2. Enter From = the safety conference's date, 09:00 (9:00 am), To = the same date, 17:00 (5:00 pm)
 3. Click 'Search'</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="31" customHeight="1">
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1532,7 +1533,8 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Location: Changi Business Park
-From/To: 14 Dec 2026 09:00-17:00</t>
+From: 14 Dec 2026, 09:00 (9:00 am)
+To: 14 Dec 2026, 17:00 (5:00 pm)</t>
         </is>
       </c>
     </row>
@@ -1680,12 +1682,12 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Choose 'Jurong Gateway' in 'Location'
-2. Enter From = the day BEFORE the training 19:00, To = the same day 20:00, and click 'Search'
-3. Change the times to 08:00-11:00 on that same day and click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+2. Enter From = the day BEFORE the training, 19:00 (7:00 pm), To = the same day, 20:00 (8:00 pm), and click 'Search'
+3. Change the times to 08:00 (8:00 am) - 11:00 (11:00 am) on that same day and click 'Search'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="71.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1694,7 +1696,8 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Location: Jurong Gateway
-From/To: 18 Oct 2026 19:00-20:00, then 08:00-11:00</t>
+From: 18 Oct 2026, 19:00 (7:00 pm); To: 18 Oct 2026, 20:00 (8:00 pm)
+then From: 18 Oct 2026, 08:00 (8:00 am); To: 18 Oct 2026, 11:00 (11:00 am)</t>
         </is>
       </c>
     </row>
@@ -1843,12 +1846,12 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Choose 'Orchard Hub' in 'Location'
-2. Enter From = 1 Mar 2027 08:00, To = 1 Mar 2027 22:00, and click 'Search'
-3. Change From to 07:59 and click 'Search'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+2. Enter From = 1 Mar 2027, 08:00 (8:00 am), To = 1 Mar 2027, 22:00 (10:00 pm), and click 'Search'
+3. Change From to 07:59 (7:59 am) and click 'Search'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1857,7 +1860,8 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Location: Orchard Hub
-From/To: 1 Mar 2027 08:00-22:00, then 07:59-22:00</t>
+From: 1 Mar 2027, 08:00 (8:00 am), then 07:59 (7:59 am)
+To: 1 Mar 2027, 22:00 (10:00 pm)</t>
         </is>
       </c>
     </row>
@@ -2004,8 +2008,8 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Enter From = 1 Mar 2027 09:00, leave 'To' empty, and click 'Search'
-2. Enter To = 1 Mar 2027 09:00 and click 'Search'</t>
+          <t>1. Enter From = 1 Mar 2027, 09:00 (9:00 am), leave 'To' empty, and click 'Search'
+2. Enter To = 1 Mar 2027, 09:00 (9:00 am) and click 'Search'</t>
         </is>
       </c>
     </row>
@@ -2017,8 +2021,8 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>From: 1 Mar 2027 09:00
-To: empty, then 1 Mar 2027 09:00</t>
+          <t>From: 1 Mar 2027, 09:00 (9:00 am)
+To: empty, then 1 Mar 2027, 09:00 (9:00 am)</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2162,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="125.5" customHeight="1">
+    <row r="4" ht="139" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2166,7 +2170,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Enter From = 1 Mar 2027 09:00, To = 1 Mar 2027 12:00
+          <t>1. Enter From = 1 Mar 2027, 09:00 (9:00 am), To = 1 Mar 2027, 12:00 (12:00 pm)
 2. Enter 100 in 'Expected attendance'
 3. Choose 'Marina Centre' in 'Location' and 'Theatre' in 'Room layout'
 4. Tick 'Step-free access' and 'Hearing induction loop' under Accessibility requirements
@@ -2176,7 +2180,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="85" customHeight="1">
+    <row r="5" ht="98.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2184,7 +2188,8 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>From/To: 1 Mar 2027 09:00-12:00
+          <t>From: 1 Mar 2027, 09:00 (9:00 am)
+To: 1 Mar 2027, 12:00 (12:00 pm)
 Expected attendance: 100
 Location: Marina Centre
 Room layout: Theatre
@@ -2354,7 +2359,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="179.5" customHeight="1">
+    <row r="6" ht="193" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2363,7 +2368,7 @@
       <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Find a venue opens with breadcrumb 'Events / EVT-000004 / Find a venue' and the subtitle 'Filled in from Straits Medical Research Symposium's requirements...'.
-From/To = its date 09:00 / 18:00; Expected attendance 200; Room layout Theatre; Location 'Any building'. Wheelchair spaces and Hearing induction loop are ticked, and so are High-density WiFi, Video conferencing suite and Livestream capability; Catering pantry is NOT ticked.
+From = 7 Dec 2026, 09:00 (9:00 am) and To = 7 Dec 2026, 18:00 (6:00 pm); Expected attendance 200; Room layout Theatre; Location 'Any building'. Wheelchair spaces and Hearing induction loop are ticked, and so are High-density WiFi, Video conferencing suite and Livestream capability; Catering pantry is NOT ticked.
 Results: Marina Auditorium (MAR-AUD), Changi Conference Centre (CBP-CONF), Marina Grand Hall (MAR-GH) - Marina Grand Hall IS listed because its booking is this event's own (compare TC08). Each card has 'Check suitability'.
 No status message appears and the event stays in Planning.</t>
         </is>

</xml_diff>

<commit_message>
SPM-40-TC15: end with a reset step so the case can be rerun
The last step runs prisma/topup-spm40-46.ts, which puts the workshop back to
Approved without a reseed, and the expected result says what that prints.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-40_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-40_Test_Cases.xlsx
@@ -2492,11 +2492,11 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Logged in as Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).
-Seed: 'SPM40 Approved Workshop' (status Approved, coordinator Daniel Tan, 30 people, Classroom, 09:00-12:00 on 25 Mar 2027, day 180 of the fixed 2026-09-26 seed) - the only Approved event in the seed. If it is missing, or already in Planning because this case was run before, run: npx tsx prisma/topup-spm40-46.ts (adds or resets it without a reseed).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="71.5" customHeight="1">
+Seed: 'SPM40 Approved Workshop' (status Approved, coordinator Daniel Tan, 30 people, Classroom, 09:00-12:00 on 25 Mar 2027, day 180 of the fixed 2026-09-26 seed) - the only Approved event in the seed. If it is missing, or still in Planning because the last run skipped the reset step, run: npx tsx prisma/topup-spm40-46.ts (adds or resets it without a reseed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="112" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2507,7 +2507,8 @@
           <t>1. Open 'SPM40 Approved Workshop' from Events and note its status badge
 2. Click the 'Venue' tab, then 'Search with filters'
 3. Go back to the event's Overview
-4. Reopen Find a venue from the Venue tab</t>
+4. Reopen Find a venue from the Venue tab
+5. Reset for the next run (this is not a reseed - it changes only this event): in the project folder run npx tsx prisma/topup-spm40-46.ts, then refresh the event's Overview</t>
         </is>
       </c>
     </row>
@@ -2523,7 +2524,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="112" customHeight="1">
+    <row r="6" ht="152.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2534,7 +2535,8 @@
           <t>Before: the status badge reads 'Approved'.
 Find a venue shows the green message 'Planning has started - This event has moved from Approved to Planning now that its venue search has begun.' above the filters, with results already listed.
 Back on the Overview the status badge reads 'Planning'.
-Reopening Find a venue shows no message and the status stays Planning.</t>
+Reopening Find a venue shows no message and the status stays Planning.
+After the reset the script prints 'SPM40 Approved Workshop: already there (was planning) - reset to approved', and the Overview's status badge reads 'Approved' again.</t>
         </is>
       </c>
     </row>

</xml_diff>